<commit_message>
Restore seven-state model and expand CWO turnover analysis
</commit_message>
<xml_diff>
--- a/observed_gene_exp.xlsx
+++ b/observed_gene_exp.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/federico/Desktop/MODEL_PAPER_GRADE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14CB488B-F1DA-574F-A06B-0EA2C614EC86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7558681-69E1-1F4A-B69A-5BEF09506474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2200" yWindow="1540" windowWidth="28040" windowHeight="17180" xr2:uid="{9B10A734-F6CD-0745-ABCC-C8F47070E311}"/>
   </bookViews>
@@ -39,29 +39,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="13">
   <si>
     <t>cwo</t>
   </si>
   <si>
-    <t>ZT0</t>
-  </si>
-  <si>
-    <t>ZT4</t>
-  </si>
-  <si>
-    <t>ZT8</t>
-  </si>
-  <si>
-    <t>ZT12</t>
-  </si>
-  <si>
-    <t>ZT16</t>
-  </si>
-  <si>
-    <t>ZT20</t>
-  </si>
-  <si>
     <t>mean</t>
   </si>
   <si>
@@ -72,6 +54,30 @@
   </si>
   <si>
     <t>per</t>
+  </si>
+  <si>
+    <t>CLK/BMAL</t>
+  </si>
+  <si>
+    <t>ZT2</t>
+  </si>
+  <si>
+    <t>ZT6</t>
+  </si>
+  <si>
+    <t>ZT10</t>
+  </si>
+  <si>
+    <t>ZT14</t>
+  </si>
+  <si>
+    <t>ZT18</t>
+  </si>
+  <si>
+    <t>ZT22</t>
+  </si>
+  <si>
+    <t>ZT26</t>
   </si>
 </sst>
 </file>
@@ -87,7 +93,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="13"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -112,11 +118,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -452,199 +461,282 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E19A2DB-93F9-8546-BB1D-1362ED82A1BE}">
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="10" max="10" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="F1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="J1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>2</v>
+      </c>
+      <c r="H2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" t="s">
+        <v>1</v>
+      </c>
+      <c r="K2" t="s">
+        <v>2</v>
+      </c>
+      <c r="L2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="2">
+        <v>1.4998519591255599</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.39560694636757598</v>
+      </c>
+      <c r="D3" s="2">
+        <v>3</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0.89880386071714002</v>
+      </c>
+      <c r="G3" s="2">
+        <v>0.10951270370098801</v>
+      </c>
+      <c r="H3" s="2">
+        <v>3</v>
+      </c>
+      <c r="J3" s="2">
+        <v>-0.97302973812293703</v>
+      </c>
+      <c r="K3" s="2">
+        <v>0.395780503790085</v>
+      </c>
+      <c r="L3" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B4" s="2">
+        <v>0.83263622036810703</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.16139201352847801</v>
+      </c>
+      <c r="D4" s="2">
+        <v>3</v>
+      </c>
+      <c r="F4" s="2">
+        <v>-0.45475685880052702</v>
+      </c>
+      <c r="G4" s="2">
+        <v>0.37367448120859598</v>
+      </c>
+      <c r="H4" s="2">
+        <v>3</v>
+      </c>
+      <c r="J4" s="2">
+        <v>-0.61634246374185497</v>
+      </c>
+      <c r="K4" s="2">
+        <v>0.348184784918454</v>
+      </c>
+      <c r="L4" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B5" s="2">
+        <v>0.60108685856815602</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0.110113006884102</v>
+      </c>
+      <c r="D5" s="2">
+        <v>3</v>
+      </c>
+      <c r="F5" s="2">
+        <v>-1.48985961556355</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0.277246082193157</v>
+      </c>
+      <c r="H5" s="2">
+        <v>3</v>
+      </c>
+      <c r="J5" s="2">
+        <v>-0.47629194658643698</v>
+      </c>
+      <c r="K5" s="2">
+        <v>1.1008130772539799</v>
+      </c>
+      <c r="L5" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="F2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="1">
-        <v>1.1446427859999999</v>
-      </c>
-      <c r="C3" s="1">
-        <v>0.18779605861073301</v>
-      </c>
-      <c r="D3" s="1">
-        <v>3</v>
-      </c>
-      <c r="F3" s="1">
-        <v>1.3725374167087701</v>
-      </c>
-      <c r="G3" s="1">
-        <v>0.12451339113711</v>
-      </c>
-      <c r="H3" s="1">
-        <v>3</v>
-      </c>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="1">
-        <v>5.9759499999999998E-3</v>
-      </c>
-      <c r="C4" s="1">
-        <v>0.13454326730093499</v>
-      </c>
-      <c r="D4" s="1">
-        <v>3</v>
-      </c>
-      <c r="F4" s="1">
-        <v>0.47572866435134897</v>
-      </c>
-      <c r="G4" s="1">
-        <v>0.20359844259833301</v>
-      </c>
-      <c r="H4" s="1">
-        <v>3</v>
-      </c>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="1">
-        <v>-1.1568946200000001</v>
-      </c>
-      <c r="C5" s="1">
-        <v>9.9228862000000001E-2</v>
-      </c>
-      <c r="D5" s="1">
-        <v>3</v>
-      </c>
-      <c r="F5" s="1">
-        <v>-0.98034767499999997</v>
-      </c>
-      <c r="G5" s="1">
-        <v>0.231444580558504</v>
-      </c>
-      <c r="H5" s="1">
-        <v>3</v>
-      </c>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="1">
-        <v>-1.2462470459999999</v>
-      </c>
-      <c r="C6" s="1">
-        <v>0.118424602416103</v>
-      </c>
-      <c r="D6" s="1">
-        <v>3</v>
-      </c>
-      <c r="F6" s="1">
-        <v>-1.3809238720000001</v>
-      </c>
-      <c r="G6" s="1">
-        <v>0.38883352742370397</v>
-      </c>
-      <c r="H6" s="1">
-        <v>3</v>
-      </c>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="1">
-        <v>-8.5712365999999998E-2</v>
-      </c>
-      <c r="C7" s="1">
-        <v>0.15245128108829001</v>
-      </c>
-      <c r="D7" s="1">
-        <v>3</v>
-      </c>
-      <c r="F7" s="1">
-        <v>-0.41065679500000002</v>
-      </c>
-      <c r="G7" s="1">
-        <v>0.294297796548803</v>
-      </c>
-      <c r="H7" s="1">
-        <v>3</v>
-      </c>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="1">
-        <v>1.3382352959999999</v>
-      </c>
-      <c r="C8" s="1">
-        <v>0.13627028109227399</v>
-      </c>
-      <c r="D8" s="1">
-        <v>3</v>
-      </c>
-      <c r="F8" s="1">
-        <v>0.92366226048931699</v>
-      </c>
-      <c r="G8" s="1">
-        <v>0.15168422781533</v>
-      </c>
-      <c r="H8" s="1">
-        <v>3</v>
-      </c>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
+      <c r="B6" s="2">
+        <v>-0.88322916339814495</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0.34850881085631003</v>
+      </c>
+      <c r="D6" s="2">
+        <v>3</v>
+      </c>
+      <c r="F6" s="2">
+        <v>-0.56875681670955802</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0.29078108138034903</v>
+      </c>
+      <c r="H6" s="2">
+        <v>3</v>
+      </c>
+      <c r="J6" s="2">
+        <v>0.61452011542214202</v>
+      </c>
+      <c r="K6" s="2">
+        <v>0.206636104687935</v>
+      </c>
+      <c r="L6" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2">
+        <v>-1.0827227281578999</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0.16958032320165001</v>
+      </c>
+      <c r="D7" s="2">
+        <v>3</v>
+      </c>
+      <c r="F7" s="2">
+        <v>-0.51207986180345799</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0.29302159288179602</v>
+      </c>
+      <c r="H7" s="2">
+        <v>3</v>
+      </c>
+      <c r="J7" s="2">
+        <v>1.5114832034196299</v>
+      </c>
+      <c r="K7" s="2">
+        <v>0.14605289739767499</v>
+      </c>
+      <c r="L7" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="2">
+        <v>9.7463006357893206E-2</v>
+      </c>
+      <c r="C8" s="2">
+        <v>0.18497309001902901</v>
+      </c>
+      <c r="D8" s="2">
+        <v>3</v>
+      </c>
+      <c r="F8" s="2">
+        <v>1.2659355683165801</v>
+      </c>
+      <c r="G8" s="2">
+        <v>0.52412081455377801</v>
+      </c>
+      <c r="H8" s="2">
+        <v>3</v>
+      </c>
+      <c r="J8" s="2">
+        <v>0.73161484962507195</v>
+      </c>
+      <c r="K8" s="2">
+        <v>0.44724557733058001</v>
+      </c>
+      <c r="L8" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="2">
+        <v>-1.0650861528636899</v>
+      </c>
+      <c r="C9" s="2">
+        <v>0.142269706030865</v>
+      </c>
+      <c r="D9" s="2">
+        <v>3</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0.86071372384336498</v>
+      </c>
+      <c r="G9" s="2">
+        <v>0.284944976668426</v>
+      </c>
+      <c r="H9" s="2">
+        <v>3</v>
+      </c>
+      <c r="J9" s="2">
+        <v>-0.79195402001561199</v>
+      </c>
+      <c r="K9" s="2">
+        <v>0.42308030224118198</v>
+      </c>
+      <c r="L9" s="2">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Update lunar phase analyses and model outputs
</commit_message>
<xml_diff>
--- a/observed_gene_exp.xlsx
+++ b/observed_gene_exp.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/federico/Desktop/MODEL_PAPER_GRADE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7558681-69E1-1F4A-B69A-5BEF09506474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F42B500-CA2A-2C45-86FC-003C66701BF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2200" yWindow="1540" windowWidth="28040" windowHeight="17180" xr2:uid="{9B10A734-F6CD-0745-ABCC-C8F47070E311}"/>
+    <workbookView xWindow="3660" yWindow="1280" windowWidth="28040" windowHeight="17180" xr2:uid="{9B10A734-F6CD-0745-ABCC-C8F47070E311}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>cwo</t>
   </si>
@@ -51,33 +51,6 @@
   </si>
   <si>
     <t>replicates</t>
-  </si>
-  <si>
-    <t>per</t>
-  </si>
-  <si>
-    <t>CLK/BMAL</t>
-  </si>
-  <si>
-    <t>ZT2</t>
-  </si>
-  <si>
-    <t>ZT6</t>
-  </si>
-  <si>
-    <t>ZT10</t>
-  </si>
-  <si>
-    <t>ZT14</t>
-  </si>
-  <si>
-    <t>ZT18</t>
-  </si>
-  <si>
-    <t>ZT22</t>
-  </si>
-  <si>
-    <t>ZT26</t>
   </si>
 </sst>
 </file>
@@ -118,15 +91,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -461,31 +435,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E19A2DB-93F9-8546-BB1D-1362ED82A1BE}">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="10" max="10" width="18.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="J1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="O1" s="3"/>
+      <c r="P1" s="3"/>
+      <c r="Q1" s="3"/>
+    </row>
+    <row r="2" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -495,254 +468,160 @@
       <c r="D2" t="s">
         <v>3</v>
       </c>
-      <c r="F2" t="s">
-        <v>1</v>
-      </c>
-      <c r="G2" t="s">
-        <v>2</v>
-      </c>
-      <c r="H2" t="s">
-        <v>3</v>
-      </c>
-      <c r="J2" t="s">
-        <v>1</v>
-      </c>
-      <c r="K2" t="s">
-        <v>2</v>
-      </c>
-      <c r="L2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+    </row>
+    <row r="3" spans="1:17" ht="17" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>3.3382200379104054E-2</v>
+      </c>
+      <c r="C3">
+        <v>0.22794383224746187</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+      <c r="Q3" s="1"/>
+    </row>
+    <row r="4" spans="1:17" ht="17" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
         <v>6</v>
       </c>
-      <c r="B3" s="2">
-        <v>1.4998519591255599</v>
-      </c>
-      <c r="C3" s="2">
-        <v>0.39560694636757598</v>
-      </c>
-      <c r="D3" s="2">
-        <v>3</v>
-      </c>
-      <c r="F3" s="2">
-        <v>0.89880386071714002</v>
-      </c>
-      <c r="G3" s="2">
-        <v>0.10951270370098801</v>
-      </c>
-      <c r="H3" s="2">
-        <v>3</v>
-      </c>
-      <c r="J3" s="2">
-        <v>-0.97302973812293703</v>
-      </c>
-      <c r="K3" s="2">
-        <v>0.395780503790085</v>
-      </c>
-      <c r="L3" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="2">
-        <v>0.83263622036810703</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0.16139201352847801</v>
-      </c>
-      <c r="D4" s="2">
-        <v>3</v>
-      </c>
-      <c r="F4" s="2">
-        <v>-0.45475685880052702</v>
-      </c>
-      <c r="G4" s="2">
-        <v>0.37367448120859598</v>
-      </c>
-      <c r="H4" s="2">
-        <v>3</v>
-      </c>
-      <c r="J4" s="2">
-        <v>-0.61634246374185497</v>
-      </c>
-      <c r="K4" s="2">
-        <v>0.348184784918454</v>
-      </c>
-      <c r="L4" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="2">
-        <v>0.60108685856815602</v>
-      </c>
-      <c r="C5" s="2">
-        <v>0.110113006884102</v>
-      </c>
-      <c r="D5" s="2">
-        <v>3</v>
-      </c>
-      <c r="F5" s="2">
-        <v>-1.48985961556355</v>
-      </c>
-      <c r="G5" s="2">
-        <v>0.277246082193157</v>
-      </c>
-      <c r="H5" s="2">
-        <v>3</v>
-      </c>
-      <c r="J5" s="2">
-        <v>-0.47629194658643698</v>
-      </c>
-      <c r="K5" s="2">
-        <v>1.1008130772539799</v>
-      </c>
-      <c r="L5" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="2">
-        <v>-0.88322916339814495</v>
-      </c>
-      <c r="C6" s="2">
-        <v>0.34850881085631003</v>
-      </c>
-      <c r="D6" s="2">
-        <v>3</v>
-      </c>
-      <c r="F6" s="2">
-        <v>-0.56875681670955802</v>
-      </c>
-      <c r="G6" s="2">
-        <v>0.29078108138034903</v>
-      </c>
-      <c r="H6" s="2">
-        <v>3</v>
-      </c>
-      <c r="J6" s="2">
-        <v>0.61452011542214202</v>
-      </c>
-      <c r="K6" s="2">
-        <v>0.206636104687935</v>
-      </c>
-      <c r="L6" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="B4">
+        <v>-0.61640621165136134</v>
+      </c>
+      <c r="C4">
+        <v>4.093992083594588E-2</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="F4" s="2"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="O4" s="1"/>
+      <c r="P4" s="1"/>
+      <c r="Q4" s="1"/>
+    </row>
+    <row r="5" spans="1:17" ht="17" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
         <v>10</v>
       </c>
-      <c r="B7" s="2">
-        <v>-1.0827227281578999</v>
-      </c>
-      <c r="C7" s="2">
-        <v>0.16958032320165001</v>
-      </c>
-      <c r="D7" s="2">
-        <v>3</v>
-      </c>
-      <c r="F7" s="2">
-        <v>-0.51207986180345799</v>
-      </c>
-      <c r="G7" s="2">
-        <v>0.29302159288179602</v>
-      </c>
-      <c r="H7" s="2">
-        <v>3</v>
-      </c>
-      <c r="J7" s="2">
-        <v>1.5114832034196299</v>
-      </c>
-      <c r="K7" s="2">
-        <v>0.14605289739767499</v>
-      </c>
-      <c r="L7" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="2">
-        <v>9.7463006357893206E-2</v>
-      </c>
-      <c r="C8" s="2">
-        <v>0.18497309001902901</v>
-      </c>
-      <c r="D8" s="2">
-        <v>3</v>
-      </c>
-      <c r="F8" s="2">
-        <v>1.2659355683165801</v>
-      </c>
-      <c r="G8" s="2">
-        <v>0.52412081455377801</v>
-      </c>
-      <c r="H8" s="2">
-        <v>3</v>
-      </c>
-      <c r="J8" s="2">
-        <v>0.73161484962507195</v>
-      </c>
-      <c r="K8" s="2">
-        <v>0.44724557733058001</v>
-      </c>
-      <c r="L8" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="2">
-        <v>-1.0650861528636899</v>
-      </c>
-      <c r="C9" s="2">
-        <v>0.142269706030865</v>
-      </c>
-      <c r="D9" s="2">
-        <v>3</v>
-      </c>
-      <c r="F9" s="2">
-        <v>0.86071372384336498</v>
-      </c>
-      <c r="G9" s="2">
-        <v>0.284944976668426</v>
-      </c>
-      <c r="H9" s="2">
-        <v>3</v>
-      </c>
-      <c r="J9" s="2">
-        <v>-0.79195402001561199</v>
-      </c>
-      <c r="K9" s="2">
-        <v>0.42308030224118198</v>
-      </c>
-      <c r="L9" s="2">
-        <v>3</v>
-      </c>
+      <c r="B5">
+        <v>-0.83998932116722036</v>
+      </c>
+      <c r="C5">
+        <v>3.301914227238107E-2</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="O5" s="1"/>
+      <c r="P5" s="1"/>
+      <c r="Q5" s="1"/>
+    </row>
+    <row r="6" spans="1:17" ht="17" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>15</v>
+      </c>
+      <c r="B6">
+        <v>-0.71189483134042619</v>
+      </c>
+      <c r="C6">
+        <v>1.8485790785421341E-2</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="1"/>
+    </row>
+    <row r="7" spans="1:17" ht="17" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>18</v>
+      </c>
+      <c r="B7">
+        <v>0.14284476441291005</v>
+      </c>
+      <c r="C7">
+        <v>0.12348044378067827</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="F7" s="2"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
+    </row>
+    <row r="8" spans="1:17" ht="17" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>22</v>
+      </c>
+      <c r="B8">
+        <v>1.9920633993669938</v>
+      </c>
+      <c r="C8">
+        <v>0.23755705386060011</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+      <c r="F8" s="2"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+    </row>
+    <row r="9" spans="1:17" ht="17" x14ac:dyDescent="0.2">
+      <c r="A9" s="2"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="J1:L1"/>
+    <mergeCell ref="O1:Q1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add configurable CWO lunar phase delay
</commit_message>
<xml_diff>
--- a/observed_gene_exp.xlsx
+++ b/observed_gene_exp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/federico/Desktop/MODEL_PAPER_GRADE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F42B500-CA2A-2C45-86FC-003C66701BF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D8CE86C-FE67-9641-BCC6-8AAF4A74BF03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3660" yWindow="1280" windowWidth="28040" windowHeight="17180" xr2:uid="{9B10A734-F6CD-0745-ABCC-C8F47070E311}"/>
+    <workbookView xWindow="1380" yWindow="1960" windowWidth="28040" windowHeight="17180" xr2:uid="{9B10A734-F6CD-0745-ABCC-C8F47070E311}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="6">
   <si>
     <t>cwo</t>
   </si>
@@ -52,12 +52,18 @@
   <si>
     <t>replicates</t>
   </si>
+  <si>
+    <t>per</t>
+  </si>
+  <si>
+    <t>clk</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -69,6 +75,14 @@
       <sz val="13"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -91,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -101,6 +115,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -435,179 +456,285 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E19A2DB-93F9-8546-BB1D-1362ED82A1BE}">
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="10.83203125" style="3"/>
     <col min="10" max="10" width="18.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
-      <c r="Q1" s="3"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="F1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="J1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
     </row>
     <row r="2" spans="1:17" ht="17" x14ac:dyDescent="0.2">
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="1"/>
+      <c r="D2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>3</v>
+      </c>
       <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
+      <c r="J2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>3</v>
+      </c>
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
     <row r="3" spans="1:17" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>3.3382200379104054E-2</v>
-      </c>
-      <c r="C3">
-        <v>0.22794383224746187</v>
+      <c r="A3" s="5">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1.1446430000000001</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.18779599999999999</v>
       </c>
       <c r="D3">
         <v>3</v>
       </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
+      <c r="F3" s="1">
+        <v>1.3725369999999999</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0.124513</v>
+      </c>
+      <c r="H3" s="1">
+        <v>3</v>
+      </c>
       <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
+      <c r="J3" s="1">
+        <v>-1.05993</v>
+      </c>
+      <c r="K3" s="1">
+        <v>0.32664700000000002</v>
+      </c>
+      <c r="L3">
+        <v>3</v>
+      </c>
       <c r="O3" s="1"/>
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
     </row>
     <row r="4" spans="1:17" ht="17" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>6</v>
-      </c>
-      <c r="B4">
-        <v>-0.61640621165136134</v>
-      </c>
-      <c r="C4">
-        <v>4.093992083594588E-2</v>
-      </c>
-      <c r="D4">
-        <v>3</v>
-      </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+      <c r="A4" s="5">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1">
+        <v>5.9760000000000004E-3</v>
+      </c>
+      <c r="C4" s="1">
+        <v>0.134543</v>
+      </c>
+      <c r="D4" s="3">
+        <v>3</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0.47572900000000001</v>
+      </c>
+      <c r="G4" s="1">
+        <v>0.203598</v>
+      </c>
+      <c r="H4" s="1">
+        <v>3</v>
+      </c>
       <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
+      <c r="J4" s="1">
+        <v>-1.145737</v>
+      </c>
+      <c r="K4" s="1">
+        <v>0.118766</v>
+      </c>
+      <c r="L4">
+        <v>3</v>
+      </c>
       <c r="O4" s="1"/>
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
     </row>
     <row r="5" spans="1:17" ht="17" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>10</v>
-      </c>
-      <c r="B5">
-        <v>-0.83998932116722036</v>
-      </c>
-      <c r="C5">
-        <v>3.301914227238107E-2</v>
-      </c>
-      <c r="D5">
-        <v>3</v>
-      </c>
-      <c r="F5" s="2"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
+      <c r="A5" s="5">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1">
+        <v>-1.156895</v>
+      </c>
+      <c r="C5" s="1">
+        <v>9.9228999999999998E-2</v>
+      </c>
+      <c r="D5" s="3">
+        <v>3</v>
+      </c>
+      <c r="F5" s="1">
+        <v>-0.980348</v>
+      </c>
+      <c r="G5" s="1">
+        <v>0.23144500000000001</v>
+      </c>
+      <c r="H5" s="1">
+        <v>3</v>
+      </c>
       <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
+      <c r="J5" s="1">
+        <v>-0.15757199999999999</v>
+      </c>
+      <c r="K5" s="1">
+        <v>4.7308000000000003E-2</v>
+      </c>
+      <c r="L5">
+        <v>3</v>
+      </c>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
     </row>
     <row r="6" spans="1:17" ht="17" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>15</v>
-      </c>
-      <c r="B6">
-        <v>-0.71189483134042619</v>
-      </c>
-      <c r="C6">
-        <v>1.8485790785421341E-2</v>
-      </c>
-      <c r="D6">
-        <v>3</v>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
+      <c r="A6" s="5">
+        <v>12</v>
+      </c>
+      <c r="B6" s="1">
+        <v>-1.2462470000000001</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0.118425</v>
+      </c>
+      <c r="D6" s="3">
+        <v>3</v>
+      </c>
+      <c r="F6" s="1">
+        <v>-1.380924</v>
+      </c>
+      <c r="G6" s="1">
+        <v>0.38883400000000001</v>
+      </c>
+      <c r="H6" s="1">
+        <v>3</v>
+      </c>
       <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
+      <c r="J6" s="1">
+        <v>1.4904090000000001</v>
+      </c>
+      <c r="K6" s="1">
+        <v>0.29412199999999999</v>
+      </c>
+      <c r="L6">
+        <v>3</v>
+      </c>
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
     </row>
     <row r="7" spans="1:17" ht="17" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>18</v>
-      </c>
-      <c r="B7">
-        <v>0.14284476441291005</v>
-      </c>
-      <c r="C7">
-        <v>0.12348044378067827</v>
-      </c>
-      <c r="D7">
-        <v>3</v>
-      </c>
-      <c r="F7" s="2"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
+      <c r="A7" s="5">
+        <v>16</v>
+      </c>
+      <c r="B7" s="1">
+        <v>-8.5711999999999997E-2</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0.152451</v>
+      </c>
+      <c r="D7" s="3">
+        <v>3</v>
+      </c>
+      <c r="F7" s="1">
+        <v>-0.41065699999999999</v>
+      </c>
+      <c r="G7" s="1">
+        <v>0.294298</v>
+      </c>
+      <c r="H7" s="1">
+        <v>3</v>
+      </c>
       <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
+      <c r="J7" s="1">
+        <v>1.1208020000000001</v>
+      </c>
+      <c r="K7" s="1">
+        <v>0.40797499999999998</v>
+      </c>
+      <c r="L7">
+        <v>3</v>
+      </c>
       <c r="O7" s="1"/>
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
     <row r="8" spans="1:17" ht="17" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>22</v>
-      </c>
-      <c r="B8">
-        <v>1.9920633993669938</v>
-      </c>
-      <c r="C8">
-        <v>0.23755705386060011</v>
-      </c>
-      <c r="D8">
-        <v>3</v>
-      </c>
-      <c r="F8" s="2"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
+      <c r="A8" s="5">
+        <v>20</v>
+      </c>
+      <c r="B8" s="1">
+        <v>1.3382350000000001</v>
+      </c>
+      <c r="C8" s="1">
+        <v>0.13627</v>
+      </c>
+      <c r="D8" s="3">
+        <v>3</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0.92366199999999998</v>
+      </c>
+      <c r="G8" s="1">
+        <v>0.15168400000000001</v>
+      </c>
+      <c r="H8" s="1">
+        <v>3</v>
+      </c>
       <c r="I8" s="1"/>
+      <c r="J8" s="1">
+        <v>-0.247972</v>
+      </c>
+      <c r="K8" s="1">
+        <v>0.63566500000000004</v>
+      </c>
+      <c r="L8">
+        <v>3</v>
+      </c>
     </row>
     <row r="9" spans="1:17" ht="17" x14ac:dyDescent="0.2">
-      <c r="A9" s="2"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
       <c r="F9" s="2"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
@@ -615,6 +742,48 @@
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="7"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18"/>
+      <c r="B18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="F18" s="4"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19"/>
+      <c r="F19" s="4"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20"/>
+      <c r="B20" s="4"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21"/>
+      <c r="B21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="F21" s="4"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22"/>
+      <c r="F22" s="4"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23"/>
+      <c r="B23" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>